<commit_message>
Execute PR #65 Grok lane: Yassir Algeria mint, Caribbean economics, decks QA
Merge PRs #58/#65 absorbed on main. Adds deterministic seal scripts for
Yassir (Morocco/Tunisia/Algeria) and Caribbean-mobility: country-reference
promotion, corridor wire, finance cascade, data-clean publish, journey relink,
and local Deck Studio validation receipts for all eleven #65 packages.
</commit_message>
<xml_diff>
--- a/finance/_refresh_bahrain-motc.xlsx
+++ b/finance/_refresh_bahrain-motc.xlsx
@@ -45,8 +45,8 @@
     <definedName name="load_sel">'Assumptions'!$B$36</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$37</definedName>
     <definedName name="country_opex">'Country opex'!$A$4:$G$4</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$97</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$97</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$96</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1814,7 +1814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX102"/>
+  <dimension ref="A1:AX101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14803,11 +14803,11 @@
       </c>
       <c r="C72" s="30" t="inlineStr">
         <is>
-          <t>Khobar / Dammam (Eastern Province) → Manama, Bahrain</t>
+          <t>Al Khor Fishing Dock → Lusail Marina Corniche</t>
         </is>
       </c>
       <c r="D72" s="31" t="n">
-        <v>18.9</v>
+        <v>20</v>
       </c>
       <c r="E72" s="26" t="n">
         <v>28</v>
@@ -14989,11 +14989,11 @@
       </c>
       <c r="C73" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Lusail Marina Corniche</t>
+          <t>Al Khor Fishing Dock → Lusail Marina Promenade</t>
         </is>
       </c>
       <c r="D73" s="31" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="E73" s="26" t="n">
         <v>28</v>
@@ -15175,11 +15175,11 @@
       </c>
       <c r="C74" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Lusail Marina Promenade</t>
+          <t>Al Khor Fishing Dock → Lusail Marina Corniche</t>
         </is>
       </c>
       <c r="D74" s="31" t="n">
-        <v>20.1</v>
+        <v>20.9</v>
       </c>
       <c r="E74" s="26" t="n">
         <v>28</v>
@@ -15361,11 +15361,11 @@
       </c>
       <c r="C75" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Lusail Marina Corniche</t>
+          <t>Manama → مرفأ صيد الخبر</t>
         </is>
       </c>
       <c r="D75" s="31" t="n">
-        <v>20.9</v>
+        <v>21</v>
       </c>
       <c r="E75" s="26" t="n">
         <v>28</v>
@@ -15547,11 +15547,11 @@
       </c>
       <c r="C76" s="30" t="inlineStr">
         <is>
-          <t>Manama → مرفأ صيد الخبر</t>
+          <t>Al Khor Fishing Dock → Marina Doha</t>
         </is>
       </c>
       <c r="D76" s="31" t="n">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="E76" s="26" t="n">
         <v>28</v>
@@ -15733,11 +15733,11 @@
       </c>
       <c r="C77" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Marina Doha</t>
+          <t>Manama → Eastern Province</t>
         </is>
       </c>
       <c r="D77" s="31" t="n">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="E77" s="26" t="n">
         <v>28</v>
@@ -15919,11 +15919,11 @@
       </c>
       <c r="C78" s="30" t="inlineStr">
         <is>
-          <t>Manama → Eastern Province</t>
+          <t>Al Khor Fishing Dock → Marina 29 @ L'encore</t>
         </is>
       </c>
       <c r="D78" s="31" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
       <c r="E78" s="26" t="n">
         <v>28</v>
@@ -16105,11 +16105,11 @@
       </c>
       <c r="C79" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Marina 29 @ L'encore</t>
+          <t>Manama → Bahrain Sailing Club</t>
         </is>
       </c>
       <c r="D79" s="31" t="n">
-        <v>21.3</v>
+        <v>22.5</v>
       </c>
       <c r="E79" s="26" t="n">
         <v>28</v>
@@ -16291,11 +16291,11 @@
       </c>
       <c r="C80" s="30" t="inlineStr">
         <is>
-          <t>Manama → Bahrain Sailing Club</t>
+          <t>Manama → Durrat Marina</t>
         </is>
       </c>
       <c r="D80" s="31" t="n">
-        <v>22.5</v>
+        <v>23.8</v>
       </c>
       <c r="E80" s="26" t="n">
         <v>28</v>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="C81" s="30" t="inlineStr">
         <is>
-          <t>Manama → Durrat Marina</t>
+          <t>Al Khor Fishing Dock → Four Seasons Luxury Marina in Doha</t>
         </is>
       </c>
       <c r="D81" s="31" t="n">
@@ -16663,11 +16663,11 @@
       </c>
       <c r="C82" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Four Seasons Luxury Marina in Doha</t>
+          <t>Manama → Marina Corniche</t>
         </is>
       </c>
       <c r="D82" s="31" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="E82" s="26" t="n">
         <v>28</v>
@@ -16849,11 +16849,11 @@
       </c>
       <c r="C83" s="30" t="inlineStr">
         <is>
-          <t>Manama → Marina Corniche</t>
+          <t>Al Khor Fishing Dock → Doha Port</t>
         </is>
       </c>
       <c r="D83" s="31" t="n">
-        <v>23.9</v>
+        <v>24.9</v>
       </c>
       <c r="E83" s="26" t="n">
         <v>28</v>
@@ -17035,11 +17035,11 @@
       </c>
       <c r="C84" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Doha Port</t>
+          <t>Manama → الارض والفضاء للترفيه البحري Land &amp; space Marina</t>
         </is>
       </c>
       <c r="D84" s="31" t="n">
-        <v>24.9</v>
+        <v>25.1</v>
       </c>
       <c r="E84" s="26" t="n">
         <v>28</v>
@@ -17221,11 +17221,11 @@
       </c>
       <c r="C85" s="30" t="inlineStr">
         <is>
-          <t>Manama → الارض والفضاء للترفيه البحري Land &amp; space Marina</t>
+          <t>Al Khor Fishing Dock → Qatar Tourist Boats</t>
         </is>
       </c>
       <c r="D85" s="31" t="n">
-        <v>25.1</v>
+        <v>26.5</v>
       </c>
       <c r="E85" s="26" t="n">
         <v>28</v>
@@ -17407,11 +17407,11 @@
       </c>
       <c r="C86" s="30" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Qatar Tourist Boats</t>
+          <t>Manama → King AbdulAziz Port - Dammam</t>
         </is>
       </c>
       <c r="D86" s="31" t="n">
-        <v>26.5</v>
+        <v>27.3</v>
       </c>
       <c r="E86" s="26" t="n">
         <v>28</v>
@@ -17593,11 +17593,11 @@
       </c>
       <c r="C87" s="30" t="inlineStr">
         <is>
-          <t>Manama → King AbdulAziz Port - Dammam</t>
+          <t>Dukhan Water Sports Club → Durrat Marina</t>
         </is>
       </c>
       <c r="D87" s="31" t="n">
-        <v>27.3</v>
+        <v>29.7</v>
       </c>
       <c r="E87" s="26" t="n">
         <v>28</v>
@@ -17779,11 +17779,11 @@
       </c>
       <c r="C88" s="30" t="inlineStr">
         <is>
-          <t>Dukhan Water Sports Club → Durrat Marina</t>
+          <t>Manama → Cornish Marina</t>
         </is>
       </c>
       <c r="D88" s="31" t="n">
-        <v>29.7</v>
+        <v>33.6</v>
       </c>
       <c r="E88" s="26" t="n">
         <v>28</v>
@@ -17965,11 +17965,11 @@
       </c>
       <c r="C89" s="30" t="inlineStr">
         <is>
-          <t>Manama → Cornish Marina</t>
+          <t>Manama → Half Moon Yacht Association</t>
         </is>
       </c>
       <c r="D89" s="31" t="n">
-        <v>33.6</v>
+        <v>36.9</v>
       </c>
       <c r="E89" s="26" t="n">
         <v>28</v>
@@ -18151,11 +18151,11 @@
       </c>
       <c r="C90" s="30" t="inlineStr">
         <is>
-          <t>Manama → Half Moon Yacht Association</t>
+          <t>Manama → Dana Bay Marina</t>
         </is>
       </c>
       <c r="D90" s="31" t="n">
-        <v>36.9</v>
+        <v>37.5</v>
       </c>
       <c r="E90" s="26" t="n">
         <v>28</v>
@@ -18325,328 +18325,142 @@
       <c r="AX90" s="44" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="29" t="inlineStr">
-        <is>
-          <t>Gulf Authority Bahrain Motc</t>
-        </is>
-      </c>
-      <c r="B91" s="29" t="inlineStr">
-        <is>
-          <t>Bahrain</t>
-        </is>
-      </c>
-      <c r="C91" s="30" t="inlineStr">
-        <is>
-          <t>Manama → Dana Bay Marina</t>
-        </is>
-      </c>
-      <c r="D91" s="31" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="E91" s="26" t="n">
-        <v>28</v>
-      </c>
-      <c r="F91" s="32" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="G91" s="32" t="inlineStr">
-        <is>
-          <t>med-low</t>
-        </is>
-      </c>
-      <c r="H91" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I91" s="33">
-        <f>60*D91/cruise_kt</f>
-        <v/>
-      </c>
-      <c r="J91" s="33">
-        <f>I91+turn_min+dwell_min</f>
-        <v/>
-      </c>
-      <c r="K91" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J91,1))</f>
-        <v/>
-      </c>
-      <c r="L91" s="34">
-        <f>ROUND(365*mech_uptime*H91,0)</f>
-        <v/>
-      </c>
-      <c r="M91" s="35">
-        <f>mech_uptime</f>
-        <v/>
-      </c>
-      <c r="N91" s="35">
-        <f>revleg_sel</f>
-        <v/>
-      </c>
-      <c r="O91" s="34">
-        <f>ROUND(K91*L91*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P91" s="36">
-        <f>load_sel</f>
-        <v/>
-      </c>
-      <c r="Q91" s="36">
-        <f>pax_cap*P91</f>
-        <v/>
-      </c>
-      <c r="R91" s="34">
-        <f>Q91*O91</f>
-        <v/>
-      </c>
-      <c r="S91" s="37">
-        <f>E91*discount</f>
-        <v/>
-      </c>
-      <c r="T91" s="38">
-        <f>S91*R91</f>
-        <v/>
-      </c>
-      <c r="U91" s="38">
-        <f>(battery/range_nm)*D91*O91*VLOOKUP(B91,country_opex,3,FALSE)</f>
-        <v/>
-      </c>
-      <c r="V91" s="38">
-        <f>VLOOKUP(B91,country_opex,2,FALSE)*crew_factor</f>
-        <v/>
-      </c>
-      <c r="W91" s="38">
-        <f>VLOOKUP(B91,country_opex,5,FALSE)</f>
-        <v/>
-      </c>
-      <c r="X91" s="38">
-        <f>maint</f>
-        <v/>
-      </c>
-      <c r="Y91" s="38">
-        <f>VLOOKUP(B91,country_opex,7,FALSE)*ins_pct</f>
-        <v/>
-      </c>
-      <c r="Z91" s="38">
-        <f>charge_berth</f>
-        <v/>
-      </c>
-      <c r="AA91" s="38">
-        <f>U91+V91+W91+X91+Y91+Z91</f>
-        <v/>
-      </c>
-      <c r="AB91" s="38">
-        <f>VLOOKUP(B91,country_opex,7,FALSE)/dep_years</f>
-        <v/>
-      </c>
-      <c r="AC91" s="38">
-        <f>T91-AA91</f>
-        <v/>
-      </c>
-      <c r="AD91" s="35">
+      <c r="A91" s="45" t="inlineStr">
+        <is>
+          <t>TOTAL / median</t>
+        </is>
+      </c>
+      <c r="T91" s="46">
+        <f>SUM(T4:T90)</f>
+        <v/>
+      </c>
+      <c r="AC91" s="46">
+        <f>SUM(AC4:AC90)</f>
+        <v/>
+      </c>
+      <c r="AD91" s="47">
         <f>IF(T91=0,"",AC91/T91)</f>
         <v/>
       </c>
-      <c r="AE91" s="36">
-        <f>IF(AC91&lt;=0,"",VLOOKUP(B91,country_opex,7,FALSE)/AC91)</f>
-        <v/>
-      </c>
-      <c r="AF91" s="33">
-        <f>((D91*O91/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D91*O91*VLOOKUP(B91,country_opex,4,FALSE))/1000</f>
-        <v/>
-      </c>
-      <c r="AG91" s="31" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AH91" s="32" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="AI91" s="32" t="inlineStr">
-        <is>
-          <t>med-low</t>
-        </is>
-      </c>
-      <c r="AJ91" s="39" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AK91" s="34">
-        <f>IF(AG91="","",AG91*AJ91)</f>
-        <v/>
-      </c>
-      <c r="AL91" s="34">
-        <f>IF(OR(AG91="",R91=0),"",MIN(IF(AS91="",9.9E+99,AS91),FLOOR(AK91/R91,1)))</f>
-        <v/>
-      </c>
-      <c r="AM91" s="38">
-        <f>IF(AL91="","",AL91*T91)</f>
-        <v/>
-      </c>
-      <c r="AN91" s="36">
-        <f>IF(OR(AG91="",R91=0),"",MIN(IF(AS91="",9.9E+99,AS91),AK91/R91))</f>
-        <v/>
-      </c>
-      <c r="AO91" s="38">
-        <f>IF(AN91="","",AN91*T91)</f>
-        <v/>
-      </c>
-      <c r="AP91" s="40" t="n"/>
-      <c r="AQ91" s="41" t="n"/>
-      <c r="AR91" s="41" t="n"/>
-      <c r="AS91" s="42" t="n"/>
-      <c r="AT91" s="43">
-        <f>IF(((S91*pax_cap*load_thin*ROUND(K91*L91*revleg_thin,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_thin,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91))&lt;=0,"",VLOOKUP(B91,country_opex,7,FALSE)/((S91*pax_cap*load_thin*ROUND(K91*L91*revleg_thin,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_thin,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91)))</f>
-        <v/>
-      </c>
-      <c r="AU91" s="43">
-        <f>IF(((S91*pax_cap*load_mid*ROUND(K91*L91*revleg_mid,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_mid,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91))&lt;=0,"",VLOOKUP(B91,country_opex,7,FALSE)/((S91*pax_cap*load_mid*ROUND(K91*L91*revleg_mid,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_mid,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91)))</f>
-        <v/>
-      </c>
-      <c r="AV91" s="43">
-        <f>IF(((S91*pax_cap*load_full*ROUND(K91*L91*revleg_full,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_full,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91))&lt;=0,"",VLOOKUP(B91,country_opex,7,FALSE)/((S91*pax_cap*load_full*ROUND(K91*L91*revleg_full,0))-(((battery/range_nm)*D91*ROUND(K91*L91*revleg_full,0)*VLOOKUP(B91,country_opex,3,FALSE))+V91+W91+X91+Y91+Z91)))</f>
-        <v/>
-      </c>
-      <c r="AW91" s="44" t="n"/>
-      <c r="AX91" s="44" t="n"/>
+      <c r="AL91" s="48">
+        <f>SUM(AL4:AL90)</f>
+        <v/>
+      </c>
+      <c r="AM91" s="46">
+        <f>SUM(AM4:AM90)</f>
+        <v/>
+      </c>
     </row>
-    <row r="92">
-      <c r="A92" s="45" t="inlineStr">
-        <is>
-          <t>TOTAL / median</t>
-        </is>
-      </c>
-      <c r="T92" s="46">
-        <f>SUM(T4:T91)</f>
-        <v/>
-      </c>
-      <c r="AC92" s="46">
-        <f>SUM(AC4:AC91)</f>
-        <v/>
-      </c>
-      <c r="AD92" s="47">
-        <f>IF(T92=0,"",AC92/T92)</f>
-        <v/>
-      </c>
-      <c r="AL92" s="48">
-        <f>SUM(AL4:AL91)</f>
-        <v/>
-      </c>
-      <c r="AM92" s="46">
-        <f>SUM(AM4:AM91)</f>
-        <v/>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
+        </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
+      <c r="A94" s="24" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B94" s="24" t="inlineStr">
+        <is>
+          <t>Fleet basis</t>
+        </is>
+      </c>
+      <c r="C94" s="24" t="inlineStr">
+        <is>
+          <t>Raw vessels (sum)</t>
+        </is>
+      </c>
+      <c r="D94" s="24" t="inlineStr">
+        <is>
+          <t>Fleet (rounded once)</t>
+        </is>
+      </c>
+      <c r="E94" s="24" t="inlineStr">
+        <is>
+          <t>Market rev/yr (raw sum)</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="24" t="inlineStr">
-        <is>
-          <t>Market</t>
-        </is>
-      </c>
-      <c r="B95" s="24" t="inlineStr">
-        <is>
-          <t>Fleet basis</t>
-        </is>
-      </c>
-      <c r="C95" s="24" t="inlineStr">
-        <is>
-          <t>Raw vessels (sum)</t>
-        </is>
-      </c>
-      <c r="D95" s="24" t="inlineStr">
-        <is>
-          <t>Fleet (rounded once)</t>
-        </is>
-      </c>
-      <c r="E95" s="24" t="inlineStr">
-        <is>
-          <t>Market rev/yr (raw sum)</t>
-        </is>
+      <c r="A95" s="25" t="inlineStr">
+        <is>
+          <t>Gulf Authority Bahrain Motc</t>
+        </is>
+      </c>
+      <c r="B95" s="13" t="inlineStr">
+        <is>
+          <t>network_sum / ceil</t>
+        </is>
+      </c>
+      <c r="C95" s="23">
+        <f>SUMIFS(AN4:AN90,A4:A90,"Gulf Authority Bahrain Motc",AP4:AP90,"=",AQ4:AQ90,"=",AR4:AR90,"=")</f>
+        <v/>
+      </c>
+      <c r="D95" s="49">
+        <f>IF(C95=0,0,CEILING(C95,1))</f>
+        <v/>
+      </c>
+      <c r="E95" s="50">
+        <f>SUMIFS(AO4:AO90,A4:A90,"Gulf Authority Bahrain Motc",AP4:AP90,"=",AQ4:AQ90,"=",AR4:AR90,"=")</f>
+        <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="25" t="inlineStr">
-        <is>
-          <t>Gulf Authority Bahrain Motc</t>
-        </is>
-      </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>network_sum / ceil</t>
-        </is>
-      </c>
-      <c r="C96" s="23">
-        <f>SUMIFS(AN4:AN91,A4:A91,"Gulf Authority Bahrain Motc",AP4:AP91,"=",AQ4:AQ91,"=",AR4:AR91,"=")</f>
-        <v/>
-      </c>
-      <c r="D96" s="49">
-        <f>IF(C96=0,0,CEILING(C96,1))</f>
-        <v/>
-      </c>
-      <c r="E96" s="50">
-        <f>SUMIFS(AO4:AO91,A4:A91,"Gulf Authority Bahrain Motc",AP4:AP91,"=",AQ4:AQ91,"=",AR4:AR91,"=")</f>
+      <c r="A96" s="45" t="inlineStr">
+        <is>
+          <t>GROUNDED FLOOR (PUBLISHED)</t>
+        </is>
+      </c>
+      <c r="D96" s="48">
+        <f>SUM(D95:D95)</f>
+        <v/>
+      </c>
+      <c r="E96" s="46">
+        <f>SUM(E95:E95)</f>
         <v/>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="45" t="inlineStr">
-        <is>
-          <t>GROUNDED FLOOR (PUBLISHED)</t>
-        </is>
-      </c>
-      <c r="D97" s="48">
-        <f>SUM(D96:D96)</f>
-        <v/>
-      </c>
-      <c r="E97" s="46">
-        <f>SUM(E96:E96)</f>
-        <v/>
+    <row r="98">
+      <c r="A98" s="51" t="inlineStr">
+        <is>
+          <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
+        </is>
+      </c>
+      <c r="C98" s="52" t="inlineStr">
+        <is>
+          <t>Al Khor Fishing Dock → Hawar Resort Hotel Jetty (88.3nm)</t>
+        </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="51" t="inlineStr">
-        <is>
-          <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
-        </is>
-      </c>
       <c r="C99" s="52" t="inlineStr">
         <is>
-          <t>Al Khor Fishing Dock → Hawar Resort Hotel Jetty (88.3nm)</t>
+          <t>Manama → Dubai (290.6nm)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="C100" s="52" t="inlineStr">
         <is>
-          <t>Lusail Marina → Bahrain Financial Harbour Marina (BFH) (72.7nm)</t>
+          <t>Abu Dhabi → Manama (264.1nm)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="C101" s="52" t="inlineStr">
         <is>
-          <t>Doha → Manama (98.3nm)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="C102" s="52" t="inlineStr">
-        <is>
-          <t>Manama → Doha (98.8nm)</t>
+          <t>Lusail Marina → Bahrain Financial Harbour Marina (BFH) (72.7nm)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A94:L94"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A93:L93"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Recalibrate utilization scenarios: mid 15 trips/day, rev-leg 0.65
Bump headline duty cycle and revenue-leg capture in vessel-constants.json
(thin 12/.55, mid 15/.65, full 18/.85). Teach aggregate.py to pass per-scenario
max_trips_per_day. Re-run full partner cascade, rebuild economics sidecar, and
republish all transparent sheets + master tracker to Drive.
</commit_message>
<xml_diff>
--- a/finance/_refresh_bahrain-motc.xlsx
+++ b/finance/_refresh_bahrain-motc.xlsx
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Cap on revenue sailings/day — ~1 sailing/70min in a 12h window; a believable on-demand premium duty cycle, not capacity-max (Jaideep 2026-06-19).</t>
+          <t>Cap on revenue sailings/day — MID headline duty cycle; thin=12 / full=18 bookends in _utilization_scenarios (Jaideep 2026-06-21).</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1603,7 @@
         <v>0.45</v>
       </c>
       <c r="C31" s="19" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         <v>0.55</v>
       </c>
       <c r="C32" s="19" t="n">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         <v>0.7</v>
       </c>
       <c r="C33" s="19" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
@@ -2186,7 +2186,7 @@
         <v/>
       </c>
       <c r="K4" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J4,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J4,1))</f>
         <v/>
       </c>
       <c r="L4" s="34">
@@ -2372,7 +2372,7 @@
         <v/>
       </c>
       <c r="K5" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J5,1))</f>
+        <f>MIN(15,FLOOR(60*service_hr/J5,1))</f>
         <v/>
       </c>
       <c r="L5" s="34">

</xml_diff>